<commit_message>
Listing bez ceny katalogowej: 29 → 30 pozycji (21375 Godzilla)
Plik odświeżony przy sprawdzaniu, czy zestawy-bez-ceny.py żyje — żyje,
i od razu złapał nowość: 21375 Godzilla (Ideas, 2026) ma podstronę
w serwisie i nie zna ceny katalogowej. Na hubie stoi więc "cena
katalogowa nieogłoszona".

karty-poza-kolejka.xlsx wrócił do wersji z gita: uruchomienie zmieniło
tam wyłącznie znacznik czasu w metadanych archiwum, dane są co do
wiersza te same (0 pozycji). Commit binarki bez zmiany danych to czysty
szum w historii.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzZ5hRoRbmYj4cURMXc2ES
</commit_message>
<xml_diff>
--- a/materialy/zestawy-bez-ceny.xlsx
+++ b/materialy/zestawy-bez-ceny.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Metodologia" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Zestawy bez ceny'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Zestawy bez ceny'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -583,300 +583,294 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>30670</t>
+          <t>21375</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Przejażdżka saniami Świętego Mikołaja</t>
+          <t>Godzilla</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>Ideas</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>2024</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>73</v>
-      </c>
-      <c r="F3" s="10" t="inlineStr"/>
+        <v>2026</v>
+      </c>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
       <c r="G3" s="10" t="inlineStr"/>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30670/</t>
+          <t>https://tylkoklocki.pl/zestaw/21375/</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>30670-1</t>
+          <t>21375-1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>30672</t>
+          <t>30670</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Steve i mała panda</t>
+          <t>Przejażdżka saniami Świętego Mikołaja</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Minecraft</t>
+          <t>Creator</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
         <v>2024</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30672/</t>
+          <t>https://tylkoklocki.pl/zestaw/30670/</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>30672-1</t>
+          <t>30670-1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>30675</t>
+          <t>30672</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Turniejowy teren szkoleniowy</t>
+          <t>Steve i mała panda</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Ninjago</t>
+          <t>Minecraft</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
         <v>2024</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="F5" s="10" t="inlineStr"/>
       <c r="G5" s="10" t="inlineStr"/>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30675/</t>
+          <t>https://tylkoklocki.pl/zestaw/30672/</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>30675-1</t>
+          <t>30672-1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>30685</t>
+          <t>30675</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Minimodel TIE Interceptor</t>
+          <t>Turniejowy teren szkoleniowy</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Star Wars</t>
+          <t>Ninjago</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
         <v>2024</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30685/</t>
+          <t>https://tylkoklocki.pl/zestaw/30675/</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>30685-1</t>
+          <t>30675-1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>30697</t>
+          <t>30685</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Buda dla psa Novy</t>
+          <t>Minimodel TIE Interceptor</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Friends</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="10" t="inlineStr"/>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30697/</t>
+          <t>https://tylkoklocki.pl/zestaw/30685/</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>30697-1</t>
+          <t>30685-1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>30700</t>
+          <t>30697</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Bitwa Arina z Dragonem</t>
+          <t>Buda dla psa Novy</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ninjago</t>
+          <t>Friends</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
         <v>2025</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30700/</t>
+          <t>https://tylkoklocki.pl/zestaw/30697/</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>30700-1</t>
+          <t>30697-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>30705</t>
+          <t>30700</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Walka w bujnej jaskini</t>
+          <t>Bitwa Arina z Dragonem</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Minecraft</t>
+          <t>Ninjago</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
         <v>2025</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F9" s="10" t="inlineStr"/>
       <c r="G9" s="10" t="inlineStr"/>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30705/</t>
+          <t>https://tylkoklocki.pl/zestaw/30700/</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>30705-1</t>
+          <t>30700-1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>30714</t>
+          <t>30705</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Rudy kot</t>
+          <t>Walka w bujnej jaskini</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Creator</t>
+          <t>Minecraft</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>79</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>tak</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30714/</t>
+          <t>https://tylkoklocki.pl/zestaw/30705/</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>30714-1</t>
+          <t>30705-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>30715</t>
+          <t>30714</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Przyjęcie urodzinowe z uroczymi zwierzątkami</t>
+          <t>Rudy kot</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -888,7 +882,7 @@
         <v>2026</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
@@ -902,24 +896,24 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30715/</t>
+          <t>https://tylkoklocki.pl/zestaw/30714/</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>30715-1</t>
+          <t>30714-1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>30717</t>
+          <t>30715</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Śmieszny halloweenowy szkielet</t>
+          <t>Przyjęcie urodzinowe z uroczymi zwierzątkami</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -931,30 +925,38 @@
         <v>2026</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>71</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="5" t="inlineStr"/>
+        <v>64</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30717/</t>
+          <t>https://tylkoklocki.pl/zestaw/30715/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>30717-1</t>
+          <t>30715-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>30718</t>
+          <t>30717</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Śnieżna przygoda Cataclaws</t>
+          <t>Śmieszny halloweenowy szkielet</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -966,120 +968,112 @@
         <v>2026</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="10" t="inlineStr"/>
       <c r="G13" s="10" t="inlineStr"/>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30718/</t>
+          <t>https://tylkoklocki.pl/zestaw/30717/</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>30718-1</t>
+          <t>30717-1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>30720</t>
+          <t>30718</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Urodzinowa potańcówka Arielki i Florka</t>
+          <t>Śnieżna przygoda Cataclaws</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Disney</t>
+          <t>Creator</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30720/</t>
+          <t>https://tylkoklocki.pl/zestaw/30718/</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>30720-1</t>
+          <t>30718-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>30722</t>
+          <t>30720</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Domek króliczka w ogrodzie</t>
+          <t>Urodzinowa potańcówka Arielki i Florka</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Friends</t>
+          <t>Disney</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>tak</t>
-        </is>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30722/</t>
+          <t>https://tylkoklocki.pl/zestaw/30720/</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>30722-1</t>
+          <t>30720-1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>30723</t>
+          <t>30722</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Samochód ninja Cole’a</t>
+          <t>Domek króliczka w ogrodzie</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Ninjago</t>
+          <t>Friends</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1093,40 +1087,40 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30723/</t>
+          <t>https://tylkoklocki.pl/zestaw/30722/</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>30723-1</t>
+          <t>30722-1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>30724</t>
+          <t>30723</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Gabinet Dumbledore’a z Harrym Potterem</t>
+          <t>Samochód ninja Cole’a</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Harry Potter</t>
+          <t>Ninjago</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1136,40 +1130,40 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30724/</t>
+          <t>https://tylkoklocki.pl/zestaw/30723/</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>30724-1</t>
+          <t>30723-1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>30728</t>
+          <t>30724</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Minimodel Brzeszczota</t>
+          <t>Gabinet Dumbledore’a z Harrym Potterem</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Star Wars</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1179,118 +1173,118 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30728/</t>
+          <t>https://tylkoklocki.pl/zestaw/30724/</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>30728-1</t>
+          <t>30724-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>30732</t>
+          <t>30728</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Potyczka Alex przy ognisku</t>
+          <t>Minimodel Brzeszczota</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Minecraft</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="F19" s="10" t="inlineStr"/>
-      <c r="G19" s="10" t="inlineStr"/>
+        <v>74</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30732/</t>
+          <t>https://tylkoklocki.pl/zestaw/30728/</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>30732-1</t>
+          <t>30728-1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>30735</t>
+          <t>30732</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Hot Rod</t>
+          <t>Potyczka Alex przy ognisku</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Technic</t>
+          <t>Minecraft</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>83</v>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>tak</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/30735/</t>
+          <t>https://tylkoklocki.pl/zestaw/30732/</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>30735-1</t>
+          <t>30732-1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>40507</t>
+          <t>30735</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>I love Billund</t>
+          <t>Hot Rod</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Ekskluzywne i promocyjne</t>
+          <t>Technic</t>
         </is>
       </c>
       <c r="D21" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>1404</v>
+        <v>83</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1300,36 +1294,36 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40507/</t>
+          <t>https://tylkoklocki.pl/zestaw/30735/</t>
         </is>
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>40507-1</t>
+          <t>30735-1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>40890</t>
+          <t>40507</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Wielkanocne dekoracje</t>
+          <t>I love Billund</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Seasonal</t>
+          <t>Ekskluzywne i promocyjne</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>312</v>
+        <v>1404</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -1343,40 +1337,40 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40890/</t>
+          <t>https://tylkoklocki.pl/zestaw/40507/</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>40890-1</t>
+          <t>40507-1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>40897</t>
+          <t>40890</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Miecz świetlny Dartha Vadera</t>
+          <t>Wielkanocne dekoracje</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Star Wars</t>
+          <t>Seasonal</t>
         </is>
       </c>
       <c r="D23" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>174</v>
+        <v>312</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -1386,40 +1380,40 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40897/</t>
+          <t>https://tylkoklocki.pl/zestaw/40890/</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>40897-1</t>
+          <t>40890-1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>40902</t>
+          <t>40897</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Hołd dla Leonarda da Vinci</t>
+          <t>Miecz świetlny Dartha Vadera</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Ekskluzywne i promocyjne</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>251</v>
+        <v>174</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1429,36 +1423,36 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40902/</t>
+          <t>https://tylkoklocki.pl/zestaw/40897/</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>40902-1</t>
+          <t>40897-1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>40910</t>
+          <t>40902</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Mistrz Rzucania Mięsem i Podniebna - figurki</t>
+          <t>Hołd dla Leonarda da Vinci</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>BrickHeadz</t>
+          <t>Ekskluzywne i promocyjne</t>
         </is>
       </c>
       <c r="D25" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>288</v>
+        <v>251</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -1472,40 +1466,40 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40910/</t>
+          <t>https://tylkoklocki.pl/zestaw/40902/</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>40910-1</t>
+          <t>40902-1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>40916</t>
+          <t>40910</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Kwiatowa ramka na zdjęcia</t>
+          <t>Mistrz Rzucania Mięsem i Podniebna - figurki</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Botanicals</t>
+          <t>BrickHeadz</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1515,40 +1509,40 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40916/</t>
+          <t>https://tylkoklocki.pl/zestaw/40910/</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>40916-1</t>
+          <t>40910-1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>40952</t>
+          <t>40916</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Zamek LEGOLAND</t>
+          <t>Kwiatowa ramka na zdjęcia</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Ekskluzywne i promocyjne</t>
+          <t>Botanicals</t>
         </is>
       </c>
       <c r="D27" s="10" t="n">
         <v>2026</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>613</v>
+        <v>310</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -1558,36 +1552,36 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/40952/</t>
+          <t>https://tylkoklocki.pl/zestaw/40916/</t>
         </is>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>40952-1</t>
+          <t>40916-1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>66813</t>
+          <t>40952</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Seria 28 – Zwierzęta – sześciopak</t>
+          <t>Zamek LEGOLAND</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Minifigurki</t>
+          <t>Ekskluzywne i promocyjne</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
         <v>2026</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>45</v>
+        <v>613</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -1601,60 +1595,103 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>https://tylkoklocki.pl/zestaw/66813/</t>
+          <t>https://tylkoklocki.pl/zestaw/40952/</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>66813-1</t>
+          <t>40952-1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
+          <t>66813</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Seria 28 – Zwierzęta – sześciopak</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Minifigurki</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>https://tylkoklocki.pl/zestaw/66813/</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>66813-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>72050</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Mario Kart - Luigi i Mach 8</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Super Mario</t>
         </is>
       </c>
-      <c r="D29" s="10" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E29" s="10" t="n">
+      <c r="D30" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E30" s="5" t="n">
         <v>2234</v>
       </c>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="G29" s="10" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>https://tylkoklocki.pl/zestaw/72050/</t>
         </is>
       </c>
-      <c r="I29" s="11" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>72050-1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I29"/>
+  <autoFilter ref="A1:I30"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -1712,6 +1749,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1798,7 +1837,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Poza ta lista jest jeszcze 681 zestawow wycofanych bez znanej ceny katalogowej. To zaszlosc historyczna - czesto nie da sie juz ustalic polskiego RRP - wiec nie traktujemy tego jako zadania do zrobienia.</t>
+          <t>Poza ta lista jest jeszcze 434 zestawow wycofanych bez znanej ceny katalogowej. To zaszlosc historyczna - czesto nie da sie juz ustalic polskiego RRP - wiec nie traktujemy tego jako zadania do zrobienia.</t>
         </is>
       </c>
     </row>

</xml_diff>